<commit_message>
Mujo: author lookup finished, 26/38 titles from VitalSource, 12 not listed; SWDE author corrected to Shawn Moore
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/memory/mujo-textbook-authors.xlsx
+++ b/memory/mujo-textbook-authors.xlsx
@@ -459,10 +459,10 @@
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="32" customWidth="1" min="7" max="7"/>
     <col width="21" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
     <col width="60" customWidth="1" min="11" max="11"/>
-    <col width="54" customWidth="1" min="12" max="12"/>
+    <col width="51" customWidth="1" min="12" max="12"/>
     <col width="29" customWidth="1" min="13" max="13"/>
     <col width="60" customWidth="1" min="14" max="14"/>
   </cols>
@@ -683,7 +683,7 @@
       <c r="K4" t="inlineStr"/>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>Pending lookup (VitalSource rate-limited 2026-10-08)</t>
+          <t>Not on VitalSource (all ISBNs checked). Ask Britt</t>
         </is>
       </c>
       <c r="M4" t="inlineStr"/>
@@ -725,7 +725,7 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>Pending lookup (VitalSource rate-limited 2026-10-08)</t>
+          <t>Not on VitalSource (all ISBNs checked). Ask Britt</t>
         </is>
       </c>
       <c r="M5" t="inlineStr"/>
@@ -1304,7 +1304,7 @@
       <c r="H16" s="2" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Shawn Moore &amp; Adam Wilkins</t>
+          <t>Shawn Moore</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1325,7 +1325,7 @@
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Second author (Adam Wilkins) read from the VitalSource URL; confirm.</t>
+          <t>VitalSource text lists Shawn Moore only, but its URL also names Adam Wilkins. Confirm.</t>
         </is>
       </c>
     </row>
@@ -1360,16 +1360,32 @@
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" s="4" t="inlineStr">
-        <is>
-          <t>Pending lookup (VitalSource rate-limited 2026-10-08)</t>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Emma Hatfield</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Public Relations Strategy and Communications, 1st edition</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>https://www.vitalsource.com/products/public-relations-and-crisis-management-emma-hatfield-v9781998798315</t>
+        </is>
+      </c>
+      <c r="L17" s="3" t="inlineStr">
+        <is>
+          <t>Found on VitalSource</t>
         </is>
       </c>
       <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>VitalSource URL says 'public-relations-and-crisis-management' (older title?).</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1402,12 +1418,24 @@
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" s="4" t="inlineStr">
-        <is>
-          <t>Pending lookup (VitalSource rate-limited 2026-10-08)</t>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>David Shaw</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Big Data Analytics and Reporting, 1st edition</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>https://www.vitalsource.com/products/big-data-analytics-reporting-david-shaw-v9781998798001</t>
+        </is>
+      </c>
+      <c r="L18" s="3" t="inlineStr">
+        <is>
+          <t>Found on VitalSource</t>
         </is>
       </c>
       <c r="M18" t="inlineStr"/>
@@ -1444,12 +1472,24 @@
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>Pending lookup (VitalSource rate-limited 2026-10-08)</t>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Rebecca Saloustros</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Writing Digital Media Content, 1st edition</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>https://www.vitalsource.com/products/writing-digital-media-content-student-39-s-manual-rebecca-saloustros-v9781988940885</t>
+        </is>
+      </c>
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>Found on VitalSource</t>
         </is>
       </c>
       <c r="M19" t="inlineStr"/>
@@ -1486,12 +1526,24 @@
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" s="4" t="inlineStr">
-        <is>
-          <t>Pending lookup (VitalSource rate-limited 2026-10-08)</t>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Emma Hatfield</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Customer Relationship Management Marketing Automation, 1st edition</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>https://www.vitalsource.com/products/customer-relationship-management-marketing-emma-hatfield-v9781988940694</t>
+        </is>
+      </c>
+      <c r="L20" s="3" t="inlineStr">
+        <is>
+          <t>Found on VitalSource</t>
         </is>
       </c>
       <c r="M20" t="inlineStr"/>
@@ -1528,12 +1580,24 @@
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" s="4" t="inlineStr">
-        <is>
-          <t>Pending lookup (VitalSource rate-limited 2026-10-08)</t>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>David Shaw</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Influencer Marketing Fundamentals, 1st edition</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>https://www.vitalsource.com/products/influencer-marketing-fundamentals-david-shaw-v9781998798278</t>
+        </is>
+      </c>
+      <c r="L21" s="3" t="inlineStr">
+        <is>
+          <t>Found on VitalSource</t>
         </is>
       </c>
       <c r="M21" t="inlineStr"/>
@@ -1574,16 +1638,32 @@
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" s="4" t="inlineStr">
-        <is>
-          <t>Pending lookup (VitalSource rate-limited 2026-10-08)</t>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>David Shaw</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Search Engine Optimization, 4th edition</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>https://www.vitalsource.com/products/search-engine-optimization-david-shaw-v9781998798155</t>
+        </is>
+      </c>
+      <c r="L22" s="3" t="inlineStr">
+        <is>
+          <t>Found on VitalSource</t>
         </is>
       </c>
       <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>4th edition (not 1st).</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1616,16 +1696,32 @@
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" s="4" t="inlineStr">
-        <is>
-          <t>Pending lookup (VitalSource rate-limited 2026-10-08)</t>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>David Shaw</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Social Media Marketing Strategies, 7th edition</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>https://www.vitalsource.com/products/social-media-marketing-strategies-david-shaw-v9781998671335</t>
+        </is>
+      </c>
+      <c r="L23" s="3" t="inlineStr">
+        <is>
+          <t>Found on VitalSource</t>
         </is>
       </c>
       <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>7th edition (not 1st).</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1658,16 +1754,32 @@
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" s="4" t="inlineStr">
-        <is>
-          <t>Pending lookup (VitalSource rate-limited 2026-10-08)</t>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>David Shaw, Alex Strauss</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Principles of Marketing, 1st edition</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>https://www.vitalsource.com/products/principles-of-marketing-david-shaw-v9781998798032</t>
+        </is>
+      </c>
+      <c r="L24" s="3" t="inlineStr">
+        <is>
+          <t>Found on VitalSource</t>
         </is>
       </c>
       <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Two authors: David Shaw and Alex Strauss (Mujo's President).</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1700,16 +1812,32 @@
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" s="4" t="inlineStr">
-        <is>
-          <t>Pending lookup (VitalSource rate-limited 2026-10-08)</t>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Shaw &amp; Wilkins</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Digital Marketing Fundamentals, 3rd edition</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>https://www.vitalsource.com/products/digital-marketing-fundamentals-shaw-amp-wilkins-v9781998798490</t>
+        </is>
+      </c>
+      <c r="L25" s="3" t="inlineStr">
+        <is>
+          <t>Found on VitalSource</t>
         </is>
       </c>
       <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>VitalSource gives surnames only ('Shaw &amp; Wilkins'). Probably David Shaw &amp; Adam Wilkins. Confirm full names.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1742,12 +1870,24 @@
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" s="4" t="inlineStr">
-        <is>
-          <t>Pending lookup (VitalSource rate-limited 2026-10-08)</t>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>David Shaw</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Prompt Engineering and LLMs, 1st edition</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>https://www.vitalsource.com/products/prompt-engineering-and-llms-david-shaw-v9781998671700</t>
+        </is>
+      </c>
+      <c r="L26" s="3" t="inlineStr">
+        <is>
+          <t>Found on VitalSource</t>
         </is>
       </c>
       <c r="M26" t="inlineStr"/>
@@ -1792,16 +1932,32 @@
           <t>9781988940625</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" s="4" t="inlineStr">
-        <is>
-          <t>Pending lookup (VitalSource rate-limited 2026-10-08)</t>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Shawn Moore</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Website Design Strategy, 1st edition</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>https://www.vitalsource.com/products/website-design-strategy-adam-wilkins-v9781988940519</t>
+        </is>
+      </c>
+      <c r="L27" s="3" t="inlineStr">
+        <is>
+          <t>Found on VitalSource</t>
         </is>
       </c>
       <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>VitalSource text lists Shawn Moore, but its URL names Adam Wilkins. Confirm. VitalSource title differs: 'Website Design Strategy'.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1842,16 +1998,32 @@
           <t>9781988940564</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" s="4" t="inlineStr">
-        <is>
-          <t>Pending lookup (VitalSource rate-limited 2026-10-08)</t>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Shawn Moore</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Online Marketing Fundamentals: High School Edition, 1st edition</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>https://www.vitalsource.com/products/online-marketing-fundamentals-adam-wilkins-v9781988940472</t>
+        </is>
+      </c>
+      <c r="L28" s="3" t="inlineStr">
+        <is>
+          <t>Found on VitalSource</t>
         </is>
       </c>
       <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>VitalSource text lists Shawn Moore, but its URL names Adam Wilkins. Confirm.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1897,7 +2069,7 @@
       <c r="K29" t="inlineStr"/>
       <c r="L29" s="4" t="inlineStr">
         <is>
-          <t>Pending lookup (VitalSource rate-limited 2026-10-08)</t>
+          <t>Not on VitalSource (all ISBNs checked). Ask Britt</t>
         </is>
       </c>
       <c r="M29" t="inlineStr"/>
@@ -1947,7 +2119,7 @@
       <c r="K30" t="inlineStr"/>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Pending lookup (VitalSource rate-limited 2026-10-08)</t>
+          <t>Not on VitalSource (all ISBNs checked). Ask Britt</t>
         </is>
       </c>
       <c r="M30" t="inlineStr"/>
@@ -1992,16 +2164,32 @@
           <t>9781988940618</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" s="4" t="inlineStr">
-        <is>
-          <t>Pending lookup (VitalSource rate-limited 2026-10-08)</t>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Rebecca Saloustros</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Creating Digital Media Content: High School Edition, 1st edition</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>https://www.vitalsource.com/products/writing-online-content-rebecca-saloustros-v9781988940496</t>
+        </is>
+      </c>
+      <c r="L31" s="3" t="inlineStr">
+        <is>
+          <t>Found on VitalSource</t>
         </is>
       </c>
       <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>VitalSource URL says 'writing-online-content' (older title?).</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2047,7 +2235,7 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>Pending lookup (VitalSource rate-limited 2026-10-08)</t>
+          <t>Not on VitalSource (all ISBNs checked). Ask Britt</t>
         </is>
       </c>
       <c r="M32" t="inlineStr"/>
@@ -2097,7 +2285,7 @@
       <c r="K33" t="inlineStr"/>
       <c r="L33" s="4" t="inlineStr">
         <is>
-          <t>Pending lookup (VitalSource rate-limited 2026-10-08)</t>
+          <t>Not on VitalSource (all ISBNs checked). Ask Britt</t>
         </is>
       </c>
       <c r="M33" t="inlineStr"/>
@@ -2147,7 +2335,7 @@
       <c r="K34" t="inlineStr"/>
       <c r="L34" s="4" t="inlineStr">
         <is>
-          <t>Pending lookup (VitalSource rate-limited 2026-10-08)</t>
+          <t>Not on VitalSource (all ISBNs checked). Ask Britt</t>
         </is>
       </c>
       <c r="M34" t="inlineStr"/>
@@ -2201,7 +2389,7 @@
       <c r="K35" t="inlineStr"/>
       <c r="L35" s="4" t="inlineStr">
         <is>
-          <t>Pending lookup (VitalSource rate-limited 2026-10-08)</t>
+          <t>Not on VitalSource (all ISBNs checked). Ask Britt</t>
         </is>
       </c>
       <c r="M35" t="inlineStr"/>
@@ -2251,7 +2439,7 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Pending lookup (VitalSource rate-limited 2026-10-08)</t>
+          <t>Not on VitalSource (all ISBNs checked). Ask Britt</t>
         </is>
       </c>
       <c r="M36" t="inlineStr"/>
@@ -2301,7 +2489,7 @@
       <c r="K37" t="inlineStr"/>
       <c r="L37" s="4" t="inlineStr">
         <is>
-          <t>Pending lookup (VitalSource rate-limited 2026-10-08)</t>
+          <t>Not on VitalSource (all ISBNs checked). Ask Britt</t>
         </is>
       </c>
       <c r="M37" t="inlineStr"/>
@@ -2355,7 +2543,7 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>Pending lookup (VitalSource rate-limited 2026-10-08)</t>
+          <t>Not on VitalSource (all ISBNs checked). Ask Britt</t>
         </is>
       </c>
       <c r="M38" t="inlineStr"/>
@@ -2409,7 +2597,7 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" s="4" t="inlineStr">
         <is>
-          <t>Pending lookup (VitalSource rate-limited 2026-10-08)</t>
+          <t>Not on VitalSource (all ISBNs checked). Ask Britt</t>
         </is>
       </c>
       <c r="M39" t="inlineStr"/>
@@ -7358,7 +7546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -7395,19 +7583,26 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Pending rows: VitalSource (Cloudflare) rate-limited after ~12 lookups. Finish slowly (one lookup every few seconds) or have Britt fill in authors.</t>
+          <t>12 titles aren't on VitalSource under any of their ISBNs (checked 2026-10-08). Britt to fill in those authors. VitalSource rate-limits fast lookups: go one every ~6 seconds.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Use in schema: author = Person (named author), publisher = Mujo Learning Systems Inc. Never use Mujo as author. See memory/mujo-context.md.</t>
+          <t>Edition: most are 1st edition, but SEO is 4th, Social Media Marketing Strategies 7th, Digital Marketing Fundamentals 3rd. Use the real edition in schema.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
+        <is>
+          <t>Use in schema: author = Person (named author), publisher = Mujo Learning Systems Inc. Never use Mujo as author. See memory/mujo-context.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Britt to confirm column M before any author goes live.</t>
         </is>

</xml_diff>